<commit_message>
UPDATE CONTROL SCHEMA AND EXCEL SAMPLE FILE ADD FRAMWORK
</commit_message>
<xml_diff>
--- a/static/templates/control_template.xlsx
+++ b/static/templates/control_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\grc_backend\static\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muttraf\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04AF2FE-0D06-4E05-943B-83F854602480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38ED5C47-399C-4D22-BB38-4BBBF3E71B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="20520" windowHeight="8880" xr2:uid="{97E48413-E1D3-4226-8DF8-5CC1902389F0}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{97E48413-E1D3-4226-8DF8-5CC1902389F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="76">
   <si>
     <t>Control Name</t>
   </si>
@@ -236,17 +236,26 @@
     <t>Control applicable</t>
   </si>
   <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>NO</t>
+    <t>Framework</t>
+  </si>
+  <si>
+    <t>NIST CSF</t>
+  </si>
+  <si>
+    <t>ISO 27001</t>
+  </si>
+  <si>
+    <t>PCI DSS</t>
+  </si>
+  <si>
+    <t>HIPAA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -377,6 +386,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -723,8 +739,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1080,13 +1097,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0404A81A-B3CE-4388-B5CD-B9B854D581D4}">
-  <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="14" width="63.109375" customWidth="1"/>
+    <col min="1" max="1" width="37.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.3125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.47265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.15625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1015625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.26171875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.20703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.05078125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="63.1015625" customWidth="1"/>
+    <col min="11" max="11" width="12.15625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5234375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.26171875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.20703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1132,8 +1162,11 @@
       <c r="O1" t="s">
         <v>70</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1162,10 +1195,13 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1194,10 +1230,13 @@
         <v>20</v>
       </c>
       <c r="O3" t="s">
-        <v>72</v>
+        <v>15</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1226,10 +1265,13 @@
         <v>18</v>
       </c>
       <c r="O4" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1258,10 +1300,13 @@
         <v>18</v>
       </c>
       <c r="O5" t="s">
+        <v>15</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -1290,10 +1335,13 @@
         <v>18</v>
       </c>
       <c r="O6" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1322,10 +1370,13 @@
         <v>18</v>
       </c>
       <c r="O7" t="s">
+        <v>15</v>
+      </c>
+      <c r="P7" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -1354,10 +1405,13 @@
         <v>20</v>
       </c>
       <c r="O8" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1389,10 +1443,13 @@
         <v>18</v>
       </c>
       <c r="O9" t="s">
-        <v>72</v>
+        <v>15</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -1421,10 +1478,13 @@
         <v>20</v>
       </c>
       <c r="O10" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>59</v>
       </c>
@@ -1453,10 +1513,13 @@
         <v>64</v>
       </c>
       <c r="O11" t="s">
-        <v>71</v>
+        <v>15</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>65</v>
       </c>
@@ -1485,10 +1548,13 @@
         <v>64</v>
       </c>
       <c r="O12" t="s">
-        <v>72</v>
+        <v>15</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>67</v>
       </c>
@@ -1517,7 +1583,10 @@
         <v>64</v>
       </c>
       <c r="O13" t="s">
-        <v>71</v>
+        <v>15</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1530,12 +1599,12 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5F9C4134-4BFF-4B02-90F1-5B02913EB081}">
           <x14:formula1>
             <xm:f>'Dropdown Options'!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:G26</xm:sqref>
+          <xm:sqref>E2:G26 O2:O13</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C97C1A39-76AF-4A1E-AB59-C23322BD0770}">
           <x14:formula1>
@@ -1549,6 +1618,12 @@
           </x14:formula1>
           <xm:sqref>M2:M26</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4FA77BB6-F5F8-496A-98AC-E3C09B5A87EC}">
+          <x14:formula1>
+            <xm:f>'Dropdown Options'!$D$2:$D$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>P2:P13</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -1557,13 +1632,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2D0213-5A52-4157-A6EC-FBBFBDFF9D10}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.68359375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1573,8 +1648,11 @@
       <c r="C1" t="s">
         <v>21</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1584,8 +1662,11 @@
       <c r="C2" t="s">
         <v>22</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1595,13 +1676,24 @@
       <c r="C3" t="s">
         <v>23</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>73</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="D5" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update control template Excel file
</commit_message>
<xml_diff>
--- a/static/templates/control_template.xlsx
+++ b/static/templates/control_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muttraf\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cydea\grc_backend\static\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38ED5C47-399C-4D22-BB38-4BBBF3E71B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74941C6-23ED-4D7C-BE07-9D093DB4E217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{97E48413-E1D3-4226-8DF8-5CC1902389F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97E48413-E1D3-4226-8DF8-5CC1902389F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -739,9 +739,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -801,9 +802,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -841,7 +842,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -947,7 +948,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1089,7 +1090,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1098,29 +1099,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0404A81A-B3CE-4388-B5CD-B9B854D581D4}">
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.1015625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.3125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.47265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.15625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1015625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.26171875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.20703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="37.05078125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="63.1015625" customWidth="1"/>
-    <col min="11" max="11" width="12.15625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.5234375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.26171875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.20703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="63.109375" customWidth="1"/>
+    <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1166,11 +1167,11 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C2" t="s">
@@ -1201,11 +1202,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C3" t="s">
@@ -1236,11 +1237,11 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C4" t="s">
@@ -1271,11 +1272,11 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C5" t="s">
@@ -1306,11 +1307,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C6" t="s">
@@ -1341,11 +1342,11 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C7" t="s">
@@ -1376,11 +1377,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C8" t="s">
@@ -1411,11 +1412,11 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C9" t="s">
@@ -1449,11 +1450,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
@@ -1484,11 +1485,11 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>59</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>60</v>
       </c>
       <c r="C11" t="s">
@@ -1519,11 +1520,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>65</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>66</v>
       </c>
       <c r="C12" t="s">
@@ -1554,11 +1555,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>67</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C13" t="s">
@@ -1633,12 +1634,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2D0213-5A52-4157-A6EC-FBBFBDFF9D10}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15.68359375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1652,7 +1653,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1680,7 +1681,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>20</v>
       </c>
@@ -1691,7 +1692,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D5" s="1" t="s">
         <v>75</v>
       </c>

</xml_diff>

<commit_message>
Refactor control handling in bulk upload and CRUD operations to ensure proper rating assignment and compliance status; update control_id to float and adjust relationship type to uppercase.
</commit_message>
<xml_diff>
--- a/static/templates/control_template.xlsx
+++ b/static/templates/control_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cydea\grc_backend\static\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F480F7-7024-48B3-AC04-83C37CCF498B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6916647C-E51D-4397-AC33-23494D2A0826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97E48413-E1D3-4226-8DF8-5CC1902389F0}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="69">
   <si>
     <t>Control Name</t>
   </si>
@@ -53,18 +53,9 @@
     <t>Next Review Date</t>
   </si>
   <si>
-    <t>Control Rating</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Compliance Status</t>
-  </si>
-  <si>
-    <t>Control Assessment</t>
-  </si>
-  <si>
     <t>Yes / No</t>
   </si>
   <si>
@@ -213,9 +204,6 @@
   </si>
   <si>
     <t>HR Procedures are not in scope of current Risk Assessment Activity</t>
-  </si>
-  <si>
-    <t>Not Applicable</t>
   </si>
   <si>
     <t>Terms and conditions of employment</t>
@@ -1089,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0404A81A-B3CE-4388-B5CD-B9B854D581D4}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
@@ -1101,14 +1089,11 @@
     <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="37" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="63.109375" customWidth="1"/>
-    <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1143,407 +1128,365 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
+        <v>63</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="M2" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="P1" s="1" t="s">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" t="s">
+        <v>12</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+      <c r="L8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L10" t="s">
+        <v>13</v>
+      </c>
+      <c r="M10" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2" t="s">
-        <v>16</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>20</v>
-      </c>
-      <c r="O3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O4" t="s">
-        <v>16</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" t="s">
-        <v>40</v>
-      </c>
-      <c r="K5" t="s">
-        <v>18</v>
-      </c>
-      <c r="O5" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>43</v>
-      </c>
-      <c r="K6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O6" t="s">
-        <v>16</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>46</v>
-      </c>
-      <c r="K7" t="s">
-        <v>18</v>
-      </c>
-      <c r="O7" t="s">
-        <v>15</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" t="s">
-        <v>49</v>
-      </c>
-      <c r="K8" t="s">
-        <v>20</v>
-      </c>
-      <c r="O8" t="s">
-        <v>16</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" t="s">
-        <v>54</v>
-      </c>
-      <c r="K9" t="s">
-        <v>18</v>
-      </c>
-      <c r="O9" t="s">
-        <v>15</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="B11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I10" t="s">
+      <c r="C11" t="s">
         <v>58</v>
       </c>
-      <c r="K10" t="s">
-        <v>20</v>
-      </c>
-      <c r="O10" t="s">
-        <v>16</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="D11" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" t="s">
         <v>60</v>
       </c>
-      <c r="C11" t="s">
+      <c r="L11" t="s">
+        <v>12</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>61</v>
       </c>
-      <c r="D11" t="s">
+      <c r="B12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" t="s">
-        <v>63</v>
-      </c>
-      <c r="K11" t="s">
-        <v>64</v>
-      </c>
-      <c r="O11" t="s">
-        <v>15</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" t="s">
+        <v>60</v>
+      </c>
+      <c r="L12" t="s">
+        <v>12</v>
+      </c>
+      <c r="M12" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C12" t="s">
-        <v>61</v>
-      </c>
-      <c r="D12" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" t="s">
-        <v>63</v>
-      </c>
-      <c r="K12" t="s">
-        <v>64</v>
-      </c>
-      <c r="O12" t="s">
-        <v>15</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1556,30 +1499,18 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5F9C4134-4BFF-4B02-90F1-5B02913EB081}">
           <x14:formula1>
             <xm:f>'Dropdown Options'!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>O2:O12 E2:G25</xm:sqref>
+          <xm:sqref>L2:L12 E2:G25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4FA77BB6-F5F8-496A-98AC-E3C09B5A87EC}">
           <x14:formula1>
             <xm:f>'Dropdown Options'!$D$2:$D$5</xm:f>
           </x14:formula1>
-          <xm:sqref>P2:P12</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C97C1A39-76AF-4A1E-AB59-C23322BD0770}">
-          <x14:formula1>
-            <xm:f>'Dropdown Options'!$B$2:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>K2:K25</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D5750B6E-D026-4903-9786-D1349777D031}">
-          <x14:formula1>
-            <xm:f>'Dropdown Options'!$C$2:$C$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>M2:M25</xm:sqref>
+          <xm:sqref>M2:M12</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1597,60 +1528,60 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D5" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>